<commit_message>
chore(qa): regenerar plantillas QA de cargas iniciales al contrato SPEC 009
Las 4 QA_cutover_*.xlsx se regeneran desde seeds/qa_integral_dataset.py::fixtures_cutover
(QA_SYNTHETIC, empresa en blanco, portables). Incorporan el contrato nuevo: incubadora v3
(CUTOVER_HATCHERY_V3) con la columna egg_origin y dos filas (internal y purchased), hoja
Catalogos con la columna source, y mortalidad presente en reproductoras. Asi la plantilla de
incubadora deja de ser v2 (que el sistema rechazaria con TEMPLATE_VERSION_UNSUPPORTED).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit/qa-integral-dataset/fixtures/QA_cutover_breeder.xlsx
+++ b/audit/qa-integral-dataset/fixtures/QA_cutover_breeder.xlsx
@@ -1291,7 +1291,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no (obligatorio)</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no (obligatorio)</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-18T03:03:40.438740+00:00</t>
+          <t>2026-10-23T10:13:29.929138+00:00</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2176,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2205,6 +2205,11 @@
           <t>parent_code</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>